<commit_message>
Add Kimi routes and simplify prompt/pdf flows
</commit_message>
<xml_diff>
--- a/data/deliverables/resume_portfolio/resume_portfolio.xlsx
+++ b/data/deliverables/resume_portfolio/resume_portfolio.xlsx
@@ -197,9 +197,7 @@
       <c r="P2">
         <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/nokia/2026-04-08/69b622b956973837413b6091/resume.md","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/nokia/2026-04-08/69b622b956973837413b6091/resume.md")</f>
       </c>
-      <c r="Q2">
-        <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/nokia/2026-04-08/69b622b956973837413b6091/resume.pdf","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/nokia/2026-04-08/69b622b956973837413b6091/resume.pdf")</f>
-      </c>
+      <c r="Q2"/>
       <c r="R2">
         <f>HYPERLINK("https://fa-evmr-saasfaprod1.fa.ocs.oraclecloud.com/hcmUI/CandidateExperience/en/job/23181/?utm_medium=jobshare&amp;src=SNS-102","https://fa-evmr-saasfaprod1.fa.ocs.oraclecloud.com/hcmUI/CandidateExperience/en/job/23181/?utm_medium=jobshare&amp;src=SNS-102")</f>
       </c>
@@ -257,9 +255,7 @@
       <c r="P3">
         <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/general-motors/2026-04-08/69ac98f42747003c3d523072/resume.md","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/general-motors/2026-04-08/69ac98f42747003c3d523072/resume.md")</f>
       </c>
-      <c r="Q3">
-        <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/general-motors/2026-04-08/69ac98f42747003c3d523072/resume.pdf","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/general-motors/2026-04-08/69ac98f42747003c3d523072/resume.pdf")</f>
-      </c>
+      <c r="Q3"/>
       <c r="R3">
         <f>HYPERLINK("https://generalmotors.wd5.myworkdayjobs.com/Careers_GM/job/Sunnyvale-California-United-States-of-America/Senior-ML-AI-Software-Engineer---Evaluation-Insights_JR-202519722?source=LinkedIn","https://generalmotors.wd5.myworkdayjobs.com/Careers_GM/job/Sunnyvale-California-United-States-of-America/Senior-ML-AI-Software-Engineer---Evaluation-Insights_JR-202519722?source=LinkedIn")</f>
       </c>
@@ -375,9 +371,7 @@
       <c r="P5">
         <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/microsoft/2026-04-08/69d650cfe63cea7a8b6685f9/resume.md","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/microsoft/2026-04-08/69d650cfe63cea7a8b6685f9/resume.md")</f>
       </c>
-      <c r="Q5">
-        <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/microsoft/2026-04-08/69d650cfe63cea7a8b6685f9/resume.pdf","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/microsoft/2026-04-08/69d650cfe63cea7a8b6685f9/resume.pdf")</f>
-      </c>
+      <c r="Q5"/>
       <c r="R5">
         <f>HYPERLINK("https://apply.careers.microsoft.com/careers/job/1970393556856000?utm_source=linkedin&amp;domain=microsoft.com&amp;src=LinkedIn","https://apply.careers.microsoft.com/careers/job/1970393556856000?utm_source=linkedin&amp;domain=microsoft.com&amp;src=LinkedIn")</f>
       </c>
@@ -517,9 +511,7 @@
       <c r="P7">
         <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/amazon/2026-04-08/699d6a6d81476f6176b63dce/resume.md","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/amazon/2026-04-08/699d6a6d81476f6176b63dce/resume.md")</f>
       </c>
-      <c r="Q7">
-        <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/amazon/2026-04-08/699d6a6d81476f6176b63dce/resume.pdf","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/amazon/2026-04-08/699d6a6d81476f6176b63dce/resume.pdf")</f>
-      </c>
+      <c r="Q7"/>
       <c r="R7">
         <f>HYPERLINK("https://www.amazon.jobs/jobs/3127822/sde-ml-engineer-frontier-ai-robotics?cmpid=SPLICX0248M&amp;utm_source=linkedin.com&amp;utm_campaign=cxro&amp;utm_medium=social_media&amp;utm_content=job_posting&amp;ss=paid","https://www.amazon.jobs/jobs/3127822/sde-ml-engineer-frontier-ai-robotics?cmpid=SPLICX0248M&amp;utm_source=linkedin.com&amp;utm_campaign=cxro&amp;utm_medium=social_media&amp;utm_content=job_posting&amp;ss=paid")</f>
       </c>
@@ -585,9 +577,7 @@
       <c r="P8">
         <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/microsoft/2026-04-08/69d6501bcfdc6132f9469623/resume.md","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/microsoft/2026-04-08/69d6501bcfdc6132f9469623/resume.md")</f>
       </c>
-      <c r="Q8">
-        <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/microsoft/2026-04-08/69d6501bcfdc6132f9469623/resume.pdf","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/microsoft/2026-04-08/69d6501bcfdc6132f9469623/resume.pdf")</f>
-      </c>
+      <c r="Q8"/>
       <c r="R8">
         <f>HYPERLINK("https://apply.careers.microsoft.com/careers/job/1970393556857255?utm_source=linkedin&amp;domain=microsoft.com&amp;src=LinkedIn","https://apply.careers.microsoft.com/careers/job/1970393556857255?utm_source=linkedin&amp;domain=microsoft.com&amp;src=LinkedIn")</f>
       </c>
@@ -653,9 +643,7 @@
       <c r="P9">
         <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/microsoft/2026-04-08/69d65016cfdc6132f946961a/resume.md","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/microsoft/2026-04-08/69d65016cfdc6132f946961a/resume.md")</f>
       </c>
-      <c r="Q9">
-        <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/microsoft/2026-04-08/69d65016cfdc6132f946961a/resume.pdf","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/microsoft/2026-04-08/69d65016cfdc6132f946961a/resume.pdf")</f>
-      </c>
+      <c r="Q9"/>
       <c r="R9">
         <f>HYPERLINK("https://apply.careers.microsoft.com/careers/job/1970393556853526?utm_source=linkedin&amp;domain=microsoft.com&amp;src=LinkedIn","https://apply.careers.microsoft.com/careers/job/1970393556853526?utm_source=linkedin&amp;domain=microsoft.com&amp;src=LinkedIn")</f>
       </c>
@@ -1011,9 +999,7 @@
       <c r="P15">
         <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/google/2026-04-08/69ba9dd95697383741406e1b/resume.md","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/google/2026-04-08/69ba9dd95697383741406e1b/resume.md")</f>
       </c>
-      <c r="Q15">
-        <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/google/2026-04-08/69ba9dd95697383741406e1b/resume.pdf","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/google/2026-04-08/69ba9dd95697383741406e1b/resume.pdf")</f>
-      </c>
+      <c r="Q15"/>
       <c r="R15">
         <f>HYPERLINK("https://careers.google.com/jobs/results/82077133681107654-software-engineer/?src=Online/LinkedIn/linkedin_us&amp;utm_source=linkedin&amp;utm_medium=jobposting&amp;utm_campaign=contract","https://careers.google.com/jobs/results/82077133681107654-software-engineer/?src=Online/LinkedIn/linkedin_us&amp;utm_source=linkedin&amp;utm_medium=jobposting&amp;utm_campaign=contract")</f>
       </c>
@@ -1079,9 +1065,7 @@
       <c r="P16">
         <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/microsoft/2026-04-08/69d64f92706f771673baa293/resume.md","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/microsoft/2026-04-08/69d64f92706f771673baa293/resume.md")</f>
       </c>
-      <c r="Q16">
-        <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/microsoft/2026-04-08/69d64f92706f771673baa293/resume.pdf","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/microsoft/2026-04-08/69d64f92706f771673baa293/resume.pdf")</f>
-      </c>
+      <c r="Q16"/>
       <c r="R16">
         <f>HYPERLINK("https://apply.careers.microsoft.com/careers/job/1970393556619657?utm_source=linkedin&amp;domain=microsoft.com&amp;src=LinkedIn","https://apply.careers.microsoft.com/careers/job/1970393556619657?utm_source=linkedin&amp;domain=microsoft.com&amp;src=LinkedIn")</f>
       </c>
@@ -1221,9 +1205,7 @@
       <c r="P18">
         <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/google/2026-04-08/69ba92be06c1ba00c54cb3d5/resume.md","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/google/2026-04-08/69ba92be06c1ba00c54cb3d5/resume.md")</f>
       </c>
-      <c r="Q18">
-        <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/google/2026-04-08/69ba92be06c1ba00c54cb3d5/resume.pdf","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/google/2026-04-08/69ba92be06c1ba00c54cb3d5/resume.pdf")</f>
-      </c>
+      <c r="Q18"/>
       <c r="R18">
         <f>HYPERLINK("https://careers.google.com/jobs/results/142994355647324870-software-engineer/?src=Online/LinkedIn/linkedin_us&amp;utm_source=linkedin&amp;utm_medium=jobposting&amp;utm_campaign=contract","https://careers.google.com/jobs/results/142994355647324870-software-engineer/?src=Online/LinkedIn/linkedin_us&amp;utm_source=linkedin&amp;utm_medium=jobposting&amp;utm_campaign=contract")</f>
       </c>
@@ -1289,9 +1271,7 @@
       <c r="P19">
         <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/ss-c-technologies/2026-04-08/69d64ba948f0c8161d2f7366/resume.md","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/ss-c-technologies/2026-04-08/69d64ba948f0c8161d2f7366/resume.md")</f>
       </c>
-      <c r="Q19">
-        <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/ss-c-technologies/2026-04-08/69d64ba948f0c8161d2f7366/resume.pdf","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/ss-c-technologies/2026-04-08/69d64ba948f0c8161d2f7366/resume.pdf")</f>
-      </c>
+      <c r="Q19"/>
       <c r="R19">
         <f>HYPERLINK("https://www.linkedin.com/jobs/view/4386975352","https://www.linkedin.com/jobs/view/4386975352")</f>
       </c>
@@ -1365,9 +1345,7 @@
       <c r="P20">
         <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/google/2026-04-08/69ba8bc25697383741402b0f/resume.md","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/google/2026-04-08/69ba8bc25697383741402b0f/resume.md")</f>
       </c>
-      <c r="Q20">
-        <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/google/2026-04-08/69ba8bc25697383741402b0f/resume.pdf","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/google/2026-04-08/69ba8bc25697383741402b0f/resume.pdf")</f>
-      </c>
+      <c r="Q20"/>
       <c r="R20">
         <f>HYPERLINK("https://careers.google.com/jobs/results/111930608938033862-software-engineer-iii/?src=Online/LinkedIn/linkedin_us&amp;utm_source=linkedin&amp;utm_medium=jobposting&amp;utm_campaign=contract","https://careers.google.com/jobs/results/111930608938033862-software-engineer-iii/?src=Online/LinkedIn/linkedin_us&amp;utm_source=linkedin&amp;utm_medium=jobposting&amp;utm_campaign=contract")</f>
       </c>
@@ -1433,9 +1411,7 @@
       <c r="P21">
         <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/garmin/2026-04-08/699dccab81476f6176b6af20/resume.md","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/garmin/2026-04-08/699dccab81476f6176b6af20/resume.md")</f>
       </c>
-      <c r="Q21">
-        <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/garmin/2026-04-08/699dccab81476f6176b6af20/resume.pdf","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/garmin/2026-04-08/699dccab81476f6176b6af20/resume.pdf")</f>
-      </c>
+      <c r="Q21"/>
       <c r="R21">
         <f>HYPERLINK("https://careers.garmin.com/jobs/18098?lang=en-us&amp;iis=Job+Board&amp;iisn=LinkedIn","https://careers.garmin.com/jobs/18098?lang=en-us&amp;iis=Job+Board&amp;iisn=LinkedIn")</f>
       </c>
@@ -1625,9 +1601,7 @@
       <c r="P24">
         <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/netjets/2026-04-08/69ba8d643b74eb1e2c887f2b/resume.md","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/netjets/2026-04-08/69ba8d643b74eb1e2c887f2b/resume.md")</f>
       </c>
-      <c r="Q24">
-        <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/netjets/2026-04-08/69ba8d643b74eb1e2c887f2b/resume.pdf","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/netjets/2026-04-08/69ba8d643b74eb1e2c887f2b/resume.pdf")</f>
-      </c>
+      <c r="Q24"/>
       <c r="R24">
         <f>HYPERLINK("https://netjets.jobs.hr.cloud.sap/us/job/Columbus-Software-Engineer-(NJUS)-OH-43219/1374174100/?feedId=386400&amp;utm_source=LinkedInJobPostings&amp;utm_campaign=NJUS_LinkedIn&amp;src=LinkedIn","https://netjets.jobs.hr.cloud.sap/us/job/Columbus-Software-Engineer-(NJUS)-OH-43219/1374174100/?feedId=386400&amp;utm_source=LinkedInJobPostings&amp;utm_campaign=NJUS_LinkedIn&amp;src=LinkedIn")</f>
       </c>
@@ -1685,9 +1659,7 @@
       <c r="P25">
         <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/ss-c-technologies/2026-04-08/69d6128ae63cea7a8b66768d/resume.md","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/ss-c-technologies/2026-04-08/69d6128ae63cea7a8b66768d/resume.md")</f>
       </c>
-      <c r="Q25">
-        <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/ss-c-technologies/2026-04-08/69d6128ae63cea7a8b66768d/resume.pdf","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/ss-c-technologies/2026-04-08/69d6128ae63cea7a8b66768d/resume.pdf")</f>
-      </c>
+      <c r="Q25"/>
       <c r="R25">
         <f>HYPERLINK("https://wd1.myworkdaysite.com/recruiting/ssctech/SSCTechnologies/job/Jacksonville-FL/Data-Scientist_R32997-1?source=LinkedIn","https://wd1.myworkdaysite.com/recruiting/ssctech/SSCTechnologies/job/Jacksonville-FL/Data-Scientist_R32997-1?source=LinkedIn")</f>
       </c>
@@ -1761,9 +1733,7 @@
       <c r="P26">
         <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/qualcomm/2026-04-08/69a504290da45516f16da9ce/resume.md","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/qualcomm/2026-04-08/69a504290da45516f16da9ce/resume.md")</f>
       </c>
-      <c r="Q26">
-        <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/qualcomm/2026-04-08/69a504290da45516f16da9ce/resume.pdf","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/qualcomm/2026-04-08/69a504290da45516f16da9ce/resume.pdf")</f>
-      </c>
+      <c r="Q26"/>
       <c r="R26">
         <f>HYPERLINK("https://careers.qualcomm.com/careers/job/446717033485?hl=en-US&amp;utm_source=linkedin&amp;domain=qualcomm.com&amp;source=APPLICANT_SOURCE-6-2","https://careers.qualcomm.com/careers/job/446717033485?hl=en-US&amp;utm_source=linkedin&amp;domain=qualcomm.com&amp;source=APPLICANT_SOURCE-6-2")</f>
       </c>
@@ -1837,9 +1807,7 @@
       <c r="P27">
         <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/google/2026-04-08/699c43cb81476f6176b4bd94/resume.md","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/google/2026-04-08/699c43cb81476f6176b4bd94/resume.md")</f>
       </c>
-      <c r="Q27">
-        <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/google/2026-04-08/699c43cb81476f6176b4bd94/resume.pdf","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/google/2026-04-08/699c43cb81476f6176b4bd94/resume.pdf")</f>
-      </c>
+      <c r="Q27"/>
       <c r="R27">
         <f>HYPERLINK("https://careers.google.com/jobs/results/124660456668177094-practice-customer-engineer/?src=Online/LinkedIn/linkedin_us&amp;utm_source=linkedin&amp;utm_medium=jobposting&amp;utm_campaign=contract","https://careers.google.com/jobs/results/124660456668177094-practice-customer-engineer/?src=Online/LinkedIn/linkedin_us&amp;utm_source=linkedin&amp;utm_medium=jobposting&amp;utm_campaign=contract")</f>
       </c>
@@ -1905,9 +1873,7 @@
       <c r="P28">
         <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/the-walt-disney-company/2026-04-08/69b2b061ae2a534885e9dc50/resume.md","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/the-walt-disney-company/2026-04-08/69b2b061ae2a534885e9dc50/resume.md")</f>
       </c>
-      <c r="Q28">
-        <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/the-walt-disney-company/2026-04-08/69b2b061ae2a534885e9dc50/resume.pdf","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/the-walt-disney-company/2026-04-08/69b2b061ae2a534885e9dc50/resume.pdf")</f>
-      </c>
+      <c r="Q28"/>
       <c r="R28">
         <f>HYPERLINK("https://www.disneycareers.com/job/-/-/391/92655058736?source=LINKEDIN_JOB_SLOTS","https://www.disneycareers.com/job/-/-/391/92655058736?source=LINKEDIN_JOB_SLOTS")</f>
       </c>
@@ -1965,9 +1931,7 @@
       <c r="P29">
         <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/kla/2026-04-08/69d58da3366bb95ba5546066/resume.md","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/kla/2026-04-08/69d58da3366bb95ba5546066/resume.md")</f>
       </c>
-      <c r="Q29">
-        <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/kla/2026-04-08/69d58da3366bb95ba5546066/resume.pdf","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/kla/2026-04-08/69d58da3366bb95ba5546066/resume.pdf")</f>
-      </c>
+      <c r="Q29"/>
       <c r="R29">
         <f>HYPERLINK("https://kla.wd1.myworkdayjobs.com/Search/job/Milpitas-CA/Software-Engineer_2634918-2?bid=370&amp;source=Job_Board_LinkedIn","https://kla.wd1.myworkdayjobs.com/Search/job/Milpitas-CA/Software-Engineer_2634918-2?bid=370&amp;source=Job_Board_LinkedIn")</f>
       </c>
@@ -2033,9 +1997,7 @@
       <c r="P30">
         <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/kla/2026-04-08/6969fa36639b452fb57ff3d1/resume.md","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/kla/2026-04-08/6969fa36639b452fb57ff3d1/resume.md")</f>
       </c>
-      <c r="Q30">
-        <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/kla/2026-04-08/6969fa36639b452fb57ff3d1/resume.pdf","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/kla/2026-04-08/6969fa36639b452fb57ff3d1/resume.pdf")</f>
-      </c>
+      <c r="Q30"/>
       <c r="R30">
         <f>HYPERLINK("https://www.linkedin.com/jobs/view/3514793139","https://www.linkedin.com/jobs/view/3514793139")</f>
       </c>
@@ -2093,9 +2055,7 @@
       <c r="P31">
         <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/amazon-web-services-aws/2026-04-08/69d6468852a5bf58001280a7/resume.md","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/amazon-web-services-aws/2026-04-08/69d6468852a5bf58001280a7/resume.md")</f>
       </c>
-      <c r="Q31">
-        <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/amazon-web-services-aws/2026-04-08/69d6468852a5bf58001280a7/resume.pdf","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/amazon-web-services-aws/2026-04-08/69d6468852a5bf58001280a7/resume.pdf")</f>
-      </c>
+      <c r="Q31"/>
       <c r="R31">
         <f>HYPERLINK("https://www.amazon.jobs/jobs/10385689/sdeii-query-processing-aurora-dsql?cmpid=SPLICX0248M&amp;utm_source=linkedin.com&amp;utm_campaign=cxro&amp;utm_medium=social_media&amp;utm_content=job_posting&amp;ss=paid","https://www.amazon.jobs/jobs/10385689/sdeii-query-processing-aurora-dsql?cmpid=SPLICX0248M&amp;utm_source=linkedin.com&amp;utm_campaign=cxro&amp;utm_medium=social_media&amp;utm_content=job_posting&amp;ss=paid")</f>
       </c>
@@ -2227,9 +2187,7 @@
       <c r="P33">
         <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/amazon/2026-04-08/69d642dc366bb95ba554bf11/resume.md","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/amazon/2026-04-08/69d642dc366bb95ba554bf11/resume.md")</f>
       </c>
-      <c r="Q33">
-        <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/amazon/2026-04-08/69d642dc366bb95ba554bf11/resume.pdf","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/amazon/2026-04-08/69d642dc366bb95ba554bf11/resume.pdf")</f>
-      </c>
+      <c r="Q33"/>
       <c r="R33">
         <f>HYPERLINK("https://www.amazon.jobs/jobs/10385654/business-intelligence-engineer-rl-analytics?cmpid=SPLICX0248M&amp;utm_source=linkedin.com&amp;utm_campaign=cxro&amp;utm_medium=social_media&amp;utm_content=job_posting&amp;ss=paid","https://www.amazon.jobs/jobs/10385654/business-intelligence-engineer-rl-analytics?cmpid=SPLICX0248M&amp;utm_source=linkedin.com&amp;utm_campaign=cxro&amp;utm_medium=social_media&amp;utm_content=job_posting&amp;ss=paid")</f>
       </c>
@@ -2287,9 +2245,7 @@
       <c r="P34">
         <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/amazon-web-services-aws/2026-04-08/69d640ea706f771673ba9fb7/resume.md","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/amazon-web-services-aws/2026-04-08/69d640ea706f771673ba9fb7/resume.md")</f>
       </c>
-      <c r="Q34">
-        <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/amazon-web-services-aws/2026-04-08/69d640ea706f771673ba9fb7/resume.pdf","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/amazon-web-services-aws/2026-04-08/69d640ea706f771673ba9fb7/resume.pdf")</f>
-      </c>
+      <c r="Q34"/>
       <c r="R34">
         <f>HYPERLINK("https://www.amazon.jobs/jobs/3206100/system-development-engineer-aws-redshift?cmpid=SPLICX0248M&amp;utm_source=linkedin.com&amp;utm_campaign=cxro&amp;utm_medium=social_media&amp;utm_content=job_posting&amp;ss=paid","https://www.amazon.jobs/jobs/3206100/system-development-engineer-aws-redshift?cmpid=SPLICX0248M&amp;utm_source=linkedin.com&amp;utm_campaign=cxro&amp;utm_medium=social_media&amp;utm_content=job_posting&amp;ss=paid")</f>
       </c>
@@ -2355,9 +2311,7 @@
       <c r="P35">
         <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/amazon-web-services-aws/2026-04-08/69d640de52a5bf5800128045/resume.md","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/amazon-web-services-aws/2026-04-08/69d640de52a5bf5800128045/resume.md")</f>
       </c>
-      <c r="Q35">
-        <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/amazon-web-services-aws/2026-04-08/69d640de52a5bf5800128045/resume.pdf","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/amazon-web-services-aws/2026-04-08/69d640de52a5bf5800128045/resume.pdf")</f>
-      </c>
+      <c r="Q35"/>
       <c r="R35">
         <f>HYPERLINK("https://www.amazon.jobs/jobs/10385675/software-development-engineer-ii--builder-experience-genai-genai-codex-?cmpid=SPLICX0248M&amp;utm_source=linkedin.com&amp;utm_campaign=cxro&amp;utm_medium=social_media&amp;utm_content=job_posting&amp;ss=paid","https://www.amazon.jobs/jobs/10385675/software-development-engineer-ii--builder-experience-genai-genai-codex-?cmpid=SPLICX0248M&amp;utm_source=linkedin.com&amp;utm_campaign=cxro&amp;utm_medium=social_media&amp;utm_content=job_posting&amp;ss=paid")</f>
       </c>
@@ -2481,9 +2435,7 @@
       <c r="P37">
         <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/amazon-web-services-aws/2026-04-08/69d640cde63cea7a8b6682f4/resume.md","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/amazon-web-services-aws/2026-04-08/69d640cde63cea7a8b6682f4/resume.md")</f>
       </c>
-      <c r="Q37">
-        <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/amazon-web-services-aws/2026-04-08/69d640cde63cea7a8b6682f4/resume.pdf","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/amazon-web-services-aws/2026-04-08/69d640cde63cea7a8b6682f4/resume.pdf")</f>
-      </c>
+      <c r="Q37"/>
       <c r="R37">
         <f>HYPERLINK("https://www.amazon.jobs/jobs/10385710/software-development-engineer-training--certifications?cmpid=SPLICX0248M&amp;utm_source=linkedin.com&amp;utm_campaign=cxro&amp;utm_medium=social_media&amp;utm_content=job_posting&amp;ss=paid","https://www.amazon.jobs/jobs/10385710/software-development-engineer-training--certifications?cmpid=SPLICX0248M&amp;utm_source=linkedin.com&amp;utm_campaign=cxro&amp;utm_medium=social_media&amp;utm_content=job_posting&amp;ss=paid")</f>
       </c>
@@ -2599,9 +2551,7 @@
       <c r="P39">
         <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/sony-interactive-entertainment/2026-04-08/698130ba49964d25b5e4135f/resume.md","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/sony-interactive-entertainment/2026-04-08/698130ba49964d25b5e4135f/resume.md")</f>
       </c>
-      <c r="Q39">
-        <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/sony-interactive-entertainment/2026-04-08/698130ba49964d25b5e4135f/resume.pdf","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/sony-interactive-entertainment/2026-04-08/698130ba49964d25b5e4135f/resume.pdf")</f>
-      </c>
+      <c r="Q39"/>
       <c r="R39">
         <f>HYPERLINK("https://boards.greenhouse.io/embed/job_app?token=5789638004&amp;utm_source=jobright","https://boards.greenhouse.io/embed/job_app?token=5789638004&amp;utm_source=jobright")</f>
       </c>
@@ -2865,9 +2815,7 @@
       <c r="P43">
         <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/intel/2026-04-08/69d63f4dcfdc6132f9469275/resume.md","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/intel/2026-04-08/69d63f4dcfdc6132f9469275/resume.md")</f>
       </c>
-      <c r="Q43">
-        <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/intel/2026-04-08/69d63f4dcfdc6132f9469275/resume.pdf","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/intel/2026-04-08/69d63f4dcfdc6132f9469275/resume.pdf")</f>
-      </c>
+      <c r="Q43"/>
       <c r="R43">
         <f>HYPERLINK("https://intel.wd1.myworkdayjobs.com/external/job/US-Arizona-Phoenix/Junior-Software-Performance-Analysis-and-Optimization-Engineer_JR0280963","https://intel.wd1.myworkdayjobs.com/external/job/US-Arizona-Phoenix/Junior-Software-Performance-Analysis-and-Optimization-Engineer_JR0280963")</f>
       </c>
@@ -3049,9 +2997,7 @@
       <c r="P46">
         <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/travelers/2026-04-08/69cc5d28366bb95ba54ef2a0/resume.md","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/travelers/2026-04-08/69cc5d28366bb95ba54ef2a0/resume.md")</f>
       </c>
-      <c r="Q46">
-        <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/travelers/2026-04-08/69cc5d28366bb95ba54ef2a0/resume.pdf","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/travelers/2026-04-08/69cc5d28366bb95ba54ef2a0/resume.pdf")</f>
-      </c>
+      <c r="Q46"/>
       <c r="R46">
         <f>HYPERLINK("https://careers.travelers.com/job/22643600/data-scientist-applied-research-hartford-ct/?source=S0791","https://careers.travelers.com/job/22643600/data-scientist-applied-research-hartford-ct/?source=S0791")</f>
       </c>
@@ -3191,9 +3137,7 @@
       <c r="P48">
         <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/snowflake/2026-04-08/699e4a4e81476f6176b73aab/resume.md","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/snowflake/2026-04-08/699e4a4e81476f6176b73aab/resume.md")</f>
       </c>
-      <c r="Q48">
-        <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/snowflake/2026-04-08/699e4a4e81476f6176b73aab/resume.pdf","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/snowflake/2026-04-08/699e4a4e81476f6176b73aab/resume.pdf")</f>
-      </c>
+      <c r="Q48"/>
       <c r="R48">
         <f>HYPERLINK("https://careers.snowflake.com/us/en/job/SNCOUSD43A772689EB407E83CE3B247592DF49EXTERNALENUS950ABC308BFB4F159BB962713C93AA5F/Software-Engineer-Frontend?utm_source=Q2P9NP2NNP&amp;utm_medium=phenom-feeds&amp;gh_src=ed5543a62","https://careers.snowflake.com/us/en/job/SNCOUSD43A772689EB407E83CE3B247592DF49EXTERNALENUS950ABC308BFB4F159BB962713C93AA5F/Software-Engineer-Frontend?utm_source=Q2P9NP2NNP&amp;utm_medium=phenom-feeds&amp;gh_src=ed5543a62")</f>
       </c>
@@ -3251,9 +3195,7 @@
       <c r="P49">
         <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/hp/2026-04-08/69d6319c706f771673ba9d05/resume.md","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/hp/2026-04-08/69d6319c706f771673ba9d05/resume.md")</f>
       </c>
-      <c r="Q49">
-        <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/hp/2026-04-08/69d6319c706f771673ba9d05/resume.pdf","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/hp/2026-04-08/69d6319c706f771673ba9d05/resume.pdf")</f>
-      </c>
+      <c r="Q49"/>
       <c r="R49">
         <f>HYPERLINK("https://HPINC.contacthr.com/151731015?src=Linkedin+Full+Feed","https://HPINC.contacthr.com/151731015?src=Linkedin+Full+Feed")</f>
       </c>
@@ -3311,9 +3253,7 @@
       <c r="P50">
         <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/paypal/2026-04-08/699e270c81476f6176b707f8/resume.md","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/paypal/2026-04-08/699e270c81476f6176b707f8/resume.md")</f>
       </c>
-      <c r="Q50">
-        <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/paypal/2026-04-08/699e270c81476f6176b707f8/resume.pdf","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/paypal/2026-04-08/699e270c81476f6176b707f8/resume.pdf")</f>
-      </c>
+      <c r="Q50"/>
       <c r="R50">
         <f>HYPERLINK("https://paypal.eightfold.ai/careers?domain=paypal.com&amp;sort_by=relevance&amp;query=R0134713&amp;Codes=W-LINKEDIN","https://paypal.eightfold.ai/careers?domain=paypal.com&amp;sort_by=relevance&amp;query=R0134713&amp;Codes=W-LINKEDIN")</f>
       </c>
@@ -3379,9 +3319,7 @@
       <c r="P51">
         <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/paypal/2026-04-08/699e256cce78e77b4fe33807/resume.md","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/paypal/2026-04-08/699e256cce78e77b4fe33807/resume.md")</f>
       </c>
-      <c r="Q51">
-        <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/paypal/2026-04-08/699e256cce78e77b4fe33807/resume.pdf","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/paypal/2026-04-08/699e256cce78e77b4fe33807/resume.pdf")</f>
-      </c>
+      <c r="Q51"/>
       <c r="R51">
         <f>HYPERLINK("https://paypal.eightfold.ai/careers?domain=paypal.com&amp;sort_by=relevance&amp;query=R0135240&amp;Codes=W-LINKEDIN","https://paypal.eightfold.ai/careers?domain=paypal.com&amp;sort_by=relevance&amp;query=R0135240&amp;Codes=W-LINKEDIN")</f>
       </c>
@@ -3447,9 +3385,7 @@
       <c r="P52">
         <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/hdr/2026-04-08/69a2c0750da45516f16c299c/resume.md","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/hdr/2026-04-08/69a2c0750da45516f16c299c/resume.md")</f>
       </c>
-      <c r="Q52">
-        <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/hdr/2026-04-08/69a2c0750da45516f16c299c/resume.pdf","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/hdr/2026-04-08/69a2c0750da45516f16c299c/resume.pdf")</f>
-      </c>
+      <c r="Q52"/>
       <c r="R52">
         <f>HYPERLINK("https://hdr.taleo.net/careersection/ex/jobdetail.ftl?job=190711&amp;lang=en&amp;src=SNS-10025","https://hdr.taleo.net/careersection/ex/jobdetail.ftl?job=190711&amp;lang=en&amp;src=SNS-10025")</f>
       </c>
@@ -3507,9 +3443,7 @@
       <c r="P53">
         <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/jpmorganchase/2026-04-08/69cc9f35cfdc6132f94112d9/resume.md","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/jpmorganchase/2026-04-08/69cc9f35cfdc6132f94112d9/resume.md")</f>
       </c>
-      <c r="Q53">
-        <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/jpmorganchase/2026-04-08/69cc9f35cfdc6132f94112d9/resume.pdf","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/jpmorganchase/2026-04-08/69cc9f35cfdc6132f94112d9/resume.pdf")</f>
-      </c>
+      <c r="Q53"/>
       <c r="R53">
         <f>HYPERLINK("https://JPMorganChase.contacthr.com/151492194","https://JPMorganChase.contacthr.com/151492194")</f>
       </c>
@@ -3633,9 +3567,7 @@
       <c r="P55">
         <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/synopsys-inc/2026-04-08/69bb8c0706c1ba00c54e14e4/resume.md","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/synopsys-inc/2026-04-08/69bb8c0706c1ba00c54e14e4/resume.md")</f>
       </c>
-      <c r="Q55">
-        <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/synopsys-inc/2026-04-08/69bb8c0706c1ba00c54e14e4/resume.pdf","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/synopsys-inc/2026-04-08/69bb8c0706c1ba00c54e14e4/resume.pdf")</f>
-      </c>
+      <c r="Q55"/>
       <c r="R55">
         <f>HYPERLINK("https://careers.synopsys.com/job/-/-/44408/90427979216","https://careers.synopsys.com/job/-/-/44408/90427979216")</f>
       </c>
@@ -3701,9 +3633,7 @@
       <c r="P56">
         <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/keysight-technologies/2026-04-08/69a213f8359fe034b1cd5272/resume.md","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/keysight-technologies/2026-04-08/69a213f8359fe034b1cd5272/resume.md")</f>
       </c>
-      <c r="Q56">
-        <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/keysight-technologies/2026-04-08/69a213f8359fe034b1cd5272/resume.pdf","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/keysight-technologies/2026-04-08/69a213f8359fe034b1cd5272/resume.pdf")</f>
-      </c>
+      <c r="Q56"/>
       <c r="R56">
         <f>HYPERLINK("https://jobs.keysight.com/jobs/51804?lang=en-us&amp;iis=LinkedIn&amp;iisn=Linkedin&amp;mode=apply","https://jobs.keysight.com/jobs/51804?lang=en-us&amp;iis=LinkedIn&amp;iisn=Linkedin&amp;mode=apply")</f>
       </c>
@@ -3769,9 +3699,7 @@
       <c r="P57">
         <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/intertek/2026-04-08/69c8e5a61818a24cd84d814a/resume.md","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/intertek/2026-04-08/69c8e5a61818a24cd84d814a/resume.md")</f>
       </c>
-      <c r="Q57">
-        <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/intertek/2026-04-08/69c8e5a61818a24cd84d814a/resume.pdf","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/intertek/2026-04-08/69c8e5a61818a24cd84d814a/resume.pdf")</f>
-      </c>
+      <c r="Q57"/>
       <c r="R57">
         <f>HYPERLINK("https://hcog.fa.em2.oraclecloud.com/hcmUI/CandidateExperience/en/job/14083/?utm_medium=jobshare","https://hcog.fa.em2.oraclecloud.com/hcmUI/CandidateExperience/en/job/14083/?utm_medium=jobshare")</f>
       </c>
@@ -3837,9 +3765,7 @@
       <c r="P58">
         <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/adobe/2026-04-08/690e2f0a221b890c2780b8ea/resume.md","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/adobe/2026-04-08/690e2f0a221b890c2780b8ea/resume.md")</f>
       </c>
-      <c r="Q58">
-        <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/adobe/2026-04-08/690e2f0a221b890c2780b8ea/resume.pdf","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/adobe/2026-04-08/690e2f0a221b890c2780b8ea/resume.pdf")</f>
-      </c>
+      <c r="Q58"/>
       <c r="R58">
         <f>HYPERLINK("https://careers.adobe.com/us/en/job/ADOBUSR162315EXTERNALENUS/Software-Development-Engineer-3?utm_source=linkedin&amp;utm_medium=phenom-feeds&amp;source=LinkedIn","https://careers.adobe.com/us/en/job/ADOBUSR162315EXTERNALENUS/Software-Development-Engineer-3?utm_source=linkedin&amp;utm_medium=phenom-feeds&amp;source=LinkedIn")</f>
       </c>
@@ -3905,9 +3831,7 @@
       <c r="P59">
         <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/tiktok/2026-04-08/69d61c52cfdc6132f9468a50/resume.md","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/tiktok/2026-04-08/69d61c52cfdc6132f9468a50/resume.md")</f>
       </c>
-      <c r="Q59">
-        <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/tiktok/2026-04-08/69d61c52cfdc6132f9468a50/resume.pdf","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/tiktok/2026-04-08/69d61c52cfdc6132f9468a50/resume.pdf")</f>
-      </c>
+      <c r="Q59"/>
       <c r="R59">
         <f>HYPERLINK("https://lifeattiktok.com/search/7553175919393802503?spread=5MWH5CQ","https://lifeattiktok.com/search/7553175919393802503?spread=5MWH5CQ")</f>
       </c>
@@ -4039,9 +3963,7 @@
       <c r="P61">
         <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/jpmorganchase/2026-04-08/69d6104ba5c9786095e4919f/resume.md","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/jpmorganchase/2026-04-08/69d6104ba5c9786095e4919f/resume.md")</f>
       </c>
-      <c r="Q61">
-        <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/jpmorganchase/2026-04-08/69d6104ba5c9786095e4919f/resume.pdf","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/jpmorganchase/2026-04-08/69d6104ba5c9786095e4919f/resume.pdf")</f>
-      </c>
+      <c r="Q61"/>
       <c r="R61">
         <f>HYPERLINK("https://JPMorganChase.contacthr.com/151731457","https://JPMorganChase.contacthr.com/151731457")</f>
       </c>
@@ -4099,9 +4021,7 @@
       <c r="P62">
         <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/jpmorganchase/2026-04-08/69d60e05cfdc6132f946857c/resume.md","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/jpmorganchase/2026-04-08/69d60e05cfdc6132f946857c/resume.md")</f>
       </c>
-      <c r="Q62">
-        <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/jpmorganchase/2026-04-08/69d60e05cfdc6132f946857c/resume.pdf","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/jpmorganchase/2026-04-08/69d60e05cfdc6132f946857c/resume.pdf")</f>
-      </c>
+      <c r="Q62"/>
       <c r="R62">
         <f>HYPERLINK("https://JPMorganChase.contacthr.com/151730357","https://JPMorganChase.contacthr.com/151730357")</f>
       </c>
@@ -4373,9 +4293,7 @@
       <c r="P66">
         <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/thermo-fisher-scientific/2026-04-08/69d5d8a0cfdc6132f946677d/resume.md","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/thermo-fisher-scientific/2026-04-08/69d5d8a0cfdc6132f946677d/resume.md")</f>
       </c>
-      <c r="Q66">
-        <f>HYPERLINK("file:///Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/thermo-fisher-scientific/2026-04-08/69d5d8a0cfdc6132f946677d/resume.pdf","/Users/jingyizhang/Documents/Playground/projects/local_job_resume_pipeline/data/deliverables/resume_portfolio/by_company/thermo-fisher-scientific/2026-04-08/69d5d8a0cfdc6132f946677d/resume.pdf")</f>
-      </c>
+      <c r="Q66"/>
       <c r="R66">
         <f>HYPERLINK("https://jobs.thermofisher.com/global/en/job/R-01345491/Data-Scientist-I?rx_ch=jobpost&amp;rx_id=7d2f6645-32af-11f1-ac04-cfc7f8abaa70&amp;rx_job=R-01345491&amp;rx_medium=post&amp;rx_paid=0&amp;rx_r=none&amp;rx_source=linkedin&amp;rx_ts=20260408T024003Z&amp;rx_vp=linkedindirectindex&amp;utm_medium=post&amp;utm_source=jobright","https://jobs.thermofisher.com/global/en/job/R-01345491/Data-Scientist-I?rx_ch=jobpost&amp;rx_id=7d2f6645-32af-11f1-ac04-cfc7f8abaa70&amp;rx_job=R-01345491&amp;rx_medium=post&amp;rx_paid=0&amp;rx_r=none&amp;rx_source=linkedin&amp;rx_ts=20260408T024003Z&amp;rx_vp=linkedindirectindex&amp;utm_medium=post&amp;utm_source=jobright")</f>
       </c>

</xml_diff>

<commit_message>
checkpoint main worktree portfolio state
</commit_message>
<xml_diff>
--- a/data/deliverables/resume_portfolio/resume_portfolio.xlsx
+++ b/data/deliverables/resume_portfolio/resume_portfolio.xlsx
@@ -1128,8 +1128,14 @@
       </c>
       <c r="L17"/>
       <c r="M17"/>
-      <c r="N17"/>
-      <c r="O17"/>
+      <c r="N17">
+        <v>88.8</v>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
       <c r="P17"/>
       <c r="Q17"/>
       <c r="R17">
@@ -1474,8 +1480,14 @@
       </c>
       <c r="L22"/>
       <c r="M22"/>
-      <c r="N22"/>
-      <c r="O22"/>
+      <c r="N22">
+        <v>93.0</v>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
       <c r="P22"/>
       <c r="Q22"/>
       <c r="R22">
@@ -2110,8 +2122,14 @@
       <c r="K32"/>
       <c r="L32"/>
       <c r="M32"/>
-      <c r="N32"/>
-      <c r="O32"/>
+      <c r="N32">
+        <v>94.6</v>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
       <c r="P32"/>
       <c r="Q32"/>
       <c r="R32">
@@ -2374,8 +2392,14 @@
       </c>
       <c r="L36"/>
       <c r="M36"/>
-      <c r="N36"/>
-      <c r="O36"/>
+      <c r="N36">
+        <v>94.2</v>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
       <c r="P36"/>
       <c r="Q36"/>
       <c r="R36">
@@ -2490,8 +2514,14 @@
       <c r="K38"/>
       <c r="L38"/>
       <c r="M38"/>
-      <c r="N38"/>
-      <c r="O38"/>
+      <c r="N38">
+        <v>93.6</v>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
       <c r="P38"/>
       <c r="Q38"/>
       <c r="R38">
@@ -2672,8 +2702,14 @@
       <c r="K41"/>
       <c r="L41"/>
       <c r="M41"/>
-      <c r="N41"/>
-      <c r="O41"/>
+      <c r="N41">
+        <v>94.0</v>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
       <c r="P41"/>
       <c r="Q41"/>
       <c r="R41">
@@ -4480,8 +4516,14 @@
       </c>
       <c r="L69"/>
       <c r="M69"/>
-      <c r="N69"/>
-      <c r="O69"/>
+      <c r="N69">
+        <v>79.0</v>
+      </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
       <c r="P69"/>
       <c r="Q69"/>
       <c r="R69">
@@ -4546,8 +4588,14 @@
       </c>
       <c r="L70"/>
       <c r="M70"/>
-      <c r="N70"/>
-      <c r="O70"/>
+      <c r="N70">
+        <v>65.2</v>
+      </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
       <c r="P70"/>
       <c r="Q70"/>
       <c r="R70">
@@ -4778,8 +4826,14 @@
       <c r="K74"/>
       <c r="L74"/>
       <c r="M74"/>
-      <c r="N74"/>
-      <c r="O74"/>
+      <c r="N74">
+        <v>93.3</v>
+      </c>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
       <c r="P74"/>
       <c r="Q74"/>
       <c r="R74">
@@ -4952,8 +5006,14 @@
       <c r="K77"/>
       <c r="L77"/>
       <c r="M77"/>
-      <c r="N77"/>
-      <c r="O77"/>
+      <c r="N77">
+        <v>85.9</v>
+      </c>
+      <c r="O77" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
       <c r="P77"/>
       <c r="Q77"/>
       <c r="R77">
@@ -5126,8 +5186,14 @@
       <c r="K80"/>
       <c r="L80"/>
       <c r="M80"/>
-      <c r="N80"/>
-      <c r="O80"/>
+      <c r="N80">
+        <v>94.8</v>
+      </c>
+      <c r="O80" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
       <c r="P80"/>
       <c r="Q80"/>
       <c r="R80">
@@ -7300,8 +7366,14 @@
       </c>
       <c r="L115"/>
       <c r="M115"/>
-      <c r="N115"/>
-      <c r="O115"/>
+      <c r="N115">
+        <v>85.5</v>
+      </c>
+      <c r="O115" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
       <c r="P115"/>
       <c r="Q115"/>
       <c r="R115">
@@ -7366,8 +7438,14 @@
       </c>
       <c r="L116"/>
       <c r="M116"/>
-      <c r="N116"/>
-      <c r="O116"/>
+      <c r="N116">
+        <v>94.0</v>
+      </c>
+      <c r="O116" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
       <c r="P116"/>
       <c r="Q116"/>
       <c r="R116">
@@ -10760,8 +10838,14 @@
       </c>
       <c r="L169"/>
       <c r="M169"/>
-      <c r="N169"/>
-      <c r="O169"/>
+      <c r="N169">
+        <v>93.6</v>
+      </c>
+      <c r="O169" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
       <c r="P169"/>
       <c r="Q169"/>
       <c r="R169">
@@ -10876,8 +10960,14 @@
       <c r="K171"/>
       <c r="L171"/>
       <c r="M171"/>
-      <c r="N171"/>
-      <c r="O171"/>
+      <c r="N171">
+        <v>78.5</v>
+      </c>
+      <c r="O171" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
       <c r="P171"/>
       <c r="Q171"/>
       <c r="R171">
@@ -11280,8 +11370,14 @@
       </c>
       <c r="L177"/>
       <c r="M177"/>
-      <c r="N177"/>
-      <c r="O177"/>
+      <c r="N177">
+        <v>93.8</v>
+      </c>
+      <c r="O177" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
       <c r="P177"/>
       <c r="Q177"/>
       <c r="R177">
@@ -11652,8 +11748,14 @@
       <c r="K183"/>
       <c r="L183"/>
       <c r="M183"/>
-      <c r="N183"/>
-      <c r="O183"/>
+      <c r="N183">
+        <v>80.8</v>
+      </c>
+      <c r="O183" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
       <c r="P183"/>
       <c r="Q183"/>
       <c r="R183">
@@ -11776,8 +11878,14 @@
       <c r="K185"/>
       <c r="L185"/>
       <c r="M185"/>
-      <c r="N185"/>
-      <c r="O185"/>
+      <c r="N185">
+        <v>86.7</v>
+      </c>
+      <c r="O185" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
       <c r="P185"/>
       <c r="Q185"/>
       <c r="R185">
@@ -14220,8 +14328,14 @@
       <c r="K223"/>
       <c r="L223"/>
       <c r="M223"/>
-      <c r="N223"/>
-      <c r="O223"/>
+      <c r="N223">
+        <v>77.5</v>
+      </c>
+      <c r="O223" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
       <c r="P223"/>
       <c r="Q223"/>
       <c r="R223">
@@ -14666,8 +14780,14 @@
       <c r="K230"/>
       <c r="L230"/>
       <c r="M230"/>
-      <c r="N230"/>
-      <c r="O230"/>
+      <c r="N230">
+        <v>82.6</v>
+      </c>
+      <c r="O230" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
       <c r="P230"/>
       <c r="Q230"/>
       <c r="R230">
@@ -15772,8 +15892,14 @@
       <c r="K247"/>
       <c r="L247"/>
       <c r="M247"/>
-      <c r="N247"/>
-      <c r="O247"/>
+      <c r="N247">
+        <v>94.6</v>
+      </c>
+      <c r="O247" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
       <c r="P247"/>
       <c r="Q247"/>
       <c r="R247">
@@ -16664,8 +16790,14 @@
       <c r="K261"/>
       <c r="L261"/>
       <c r="M261"/>
-      <c r="N261"/>
-      <c r="O261"/>
+      <c r="N261">
+        <v>93.2</v>
+      </c>
+      <c r="O261" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
       <c r="P261"/>
       <c r="Q261"/>
       <c r="R261">
@@ -17392,8 +17524,14 @@
       <c r="K273"/>
       <c r="L273"/>
       <c r="M273"/>
-      <c r="N273"/>
-      <c r="O273"/>
+      <c r="N273">
+        <v>93.8</v>
+      </c>
+      <c r="O273" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
       <c r="P273"/>
       <c r="Q273"/>
       <c r="R273">
@@ -19160,8 +19298,14 @@
       <c r="K301"/>
       <c r="L301"/>
       <c r="M301"/>
-      <c r="N301"/>
-      <c r="O301"/>
+      <c r="N301">
+        <v>96.2</v>
+      </c>
+      <c r="O301" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
       <c r="P301"/>
       <c r="Q301"/>
       <c r="R301">
@@ -19392,8 +19536,14 @@
       <c r="K305"/>
       <c r="L305"/>
       <c r="M305"/>
-      <c r="N305"/>
-      <c r="O305"/>
+      <c r="N305">
+        <v>88.9</v>
+      </c>
+      <c r="O305" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
       <c r="P305"/>
       <c r="Q305"/>
       <c r="R305">
@@ -19508,8 +19658,14 @@
       <c r="K307"/>
       <c r="L307"/>
       <c r="M307"/>
-      <c r="N307"/>
-      <c r="O307"/>
+      <c r="N307">
+        <v>94.3</v>
+      </c>
+      <c r="O307" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
       <c r="P307"/>
       <c r="Q307"/>
       <c r="R307">
@@ -20160,8 +20316,14 @@
       <c r="K317"/>
       <c r="L317"/>
       <c r="M317"/>
-      <c r="N317"/>
-      <c r="O317"/>
+      <c r="N317">
+        <v>95.0</v>
+      </c>
+      <c r="O317" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
       <c r="P317"/>
       <c r="Q317"/>
       <c r="R317">
@@ -22076,8 +22238,14 @@
       <c r="K347"/>
       <c r="L347"/>
       <c r="M347"/>
-      <c r="N347"/>
-      <c r="O347"/>
+      <c r="N347">
+        <v>93.1</v>
+      </c>
+      <c r="O347" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
       <c r="P347"/>
       <c r="Q347"/>
       <c r="R347">
@@ -25676,8 +25844,14 @@
       <c r="K403"/>
       <c r="L403"/>
       <c r="M403"/>
-      <c r="N403"/>
-      <c r="O403"/>
+      <c r="N403">
+        <v>74.2</v>
+      </c>
+      <c r="O403" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
       <c r="P403"/>
       <c r="Q403"/>
       <c r="R403">
@@ -26064,8 +26238,14 @@
       </c>
       <c r="L409"/>
       <c r="M409"/>
-      <c r="N409"/>
-      <c r="O409"/>
+      <c r="N409">
+        <v>93.9</v>
+      </c>
+      <c r="O409" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
       <c r="P409"/>
       <c r="Q409"/>
       <c r="R409">
@@ -26436,8 +26616,14 @@
       <c r="K415"/>
       <c r="L415"/>
       <c r="M415"/>
-      <c r="N415"/>
-      <c r="O415"/>
+      <c r="N415">
+        <v>95.0</v>
+      </c>
+      <c r="O415" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
       <c r="P415"/>
       <c r="Q415"/>
       <c r="R415">
@@ -26940,8 +27126,14 @@
       <c r="K423"/>
       <c r="L423"/>
       <c r="M423"/>
-      <c r="N423"/>
-      <c r="O423"/>
+      <c r="N423">
+        <v>92.6</v>
+      </c>
+      <c r="O423" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
       <c r="P423"/>
       <c r="Q423"/>
       <c r="R423">
@@ -26998,8 +27190,14 @@
       <c r="K424"/>
       <c r="L424"/>
       <c r="M424"/>
-      <c r="N424"/>
-      <c r="O424"/>
+      <c r="N424">
+        <v>94.1</v>
+      </c>
+      <c r="O424" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
       <c r="P424"/>
       <c r="Q424"/>
       <c r="R424">
@@ -29534,8 +29732,14 @@
       <c r="K464"/>
       <c r="L464"/>
       <c r="M464"/>
-      <c r="N464"/>
-      <c r="O464"/>
+      <c r="N464">
+        <v>82.7</v>
+      </c>
+      <c r="O464" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
       <c r="P464"/>
       <c r="Q464"/>
       <c r="R464">
@@ -29880,8 +30084,14 @@
       <c r="K469"/>
       <c r="L469"/>
       <c r="M469"/>
-      <c r="N469"/>
-      <c r="O469"/>
+      <c r="N469">
+        <v>95.0</v>
+      </c>
+      <c r="O469" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
       <c r="P469"/>
       <c r="Q469"/>
       <c r="R469">
@@ -29938,8 +30148,14 @@
       <c r="K470"/>
       <c r="L470"/>
       <c r="M470"/>
-      <c r="N470"/>
-      <c r="O470"/>
+      <c r="N470">
+        <v>90.7</v>
+      </c>
+      <c r="O470" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
       <c r="P470"/>
       <c r="Q470"/>
       <c r="R470">
@@ -29996,8 +30212,14 @@
       <c r="K471"/>
       <c r="L471"/>
       <c r="M471"/>
-      <c r="N471"/>
-      <c r="O471"/>
+      <c r="N471">
+        <v>92.7</v>
+      </c>
+      <c r="O471" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
       <c r="P471"/>
       <c r="Q471"/>
       <c r="R471">
@@ -30170,8 +30392,14 @@
       <c r="K474"/>
       <c r="L474"/>
       <c r="M474"/>
-      <c r="N474"/>
-      <c r="O474"/>
+      <c r="N474">
+        <v>94.5</v>
+      </c>
+      <c r="O474" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
       <c r="P474"/>
       <c r="Q474"/>
       <c r="R474">
@@ -31086,8 +31314,14 @@
       <c r="K488"/>
       <c r="L488"/>
       <c r="M488"/>
-      <c r="N488"/>
-      <c r="O488"/>
+      <c r="N488">
+        <v>84.8</v>
+      </c>
+      <c r="O488" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
       <c r="P488"/>
       <c r="Q488"/>
       <c r="R488">
@@ -34018,8 +34252,14 @@
       <c r="K534"/>
       <c r="L534"/>
       <c r="M534"/>
-      <c r="N534"/>
-      <c r="O534"/>
+      <c r="N534">
+        <v>93.6</v>
+      </c>
+      <c r="O534" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
       <c r="P534"/>
       <c r="Q534"/>
       <c r="R534">
@@ -34084,8 +34324,14 @@
       </c>
       <c r="L535"/>
       <c r="M535"/>
-      <c r="N535"/>
-      <c r="O535"/>
+      <c r="N535">
+        <v>83.4</v>
+      </c>
+      <c r="O535" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
       <c r="P535"/>
       <c r="Q535"/>
       <c r="R535">
@@ -35520,8 +35766,14 @@
       <c r="K557"/>
       <c r="L557"/>
       <c r="M557"/>
-      <c r="N557"/>
-      <c r="O557"/>
+      <c r="N557">
+        <v>84.8</v>
+      </c>
+      <c r="O557" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
       <c r="P557"/>
       <c r="Q557"/>
       <c r="R557">
@@ -35776,8 +36028,14 @@
       <c r="K561"/>
       <c r="L561"/>
       <c r="M561"/>
-      <c r="N561"/>
-      <c r="O561"/>
+      <c r="N561">
+        <v>85.9</v>
+      </c>
+      <c r="O561" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
       <c r="P561"/>
       <c r="Q561"/>
       <c r="R561">
@@ -38658,8 +38916,14 @@
       </c>
       <c r="L606"/>
       <c r="M606"/>
-      <c r="N606"/>
-      <c r="O606"/>
+      <c r="N606">
+        <v>94.4</v>
+      </c>
+      <c r="O606" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
       <c r="P606"/>
       <c r="Q606"/>
       <c r="R606">
@@ -41886,8 +42150,14 @@
       <c r="K656"/>
       <c r="L656"/>
       <c r="M656"/>
-      <c r="N656"/>
-      <c r="O656"/>
+      <c r="N656">
+        <v>88.4</v>
+      </c>
+      <c r="O656" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
       <c r="P656"/>
       <c r="Q656"/>
       <c r="R656">
@@ -41952,8 +42222,14 @@
       </c>
       <c r="L657"/>
       <c r="M657"/>
-      <c r="N657"/>
-      <c r="O657"/>
+      <c r="N657">
+        <v>89.2</v>
+      </c>
+      <c r="O657" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
       <c r="P657"/>
       <c r="Q657"/>
       <c r="R657">
@@ -42018,8 +42294,14 @@
       </c>
       <c r="L658"/>
       <c r="M658"/>
-      <c r="N658"/>
-      <c r="O658"/>
+      <c r="N658">
+        <v>94.3</v>
+      </c>
+      <c r="O658" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
       <c r="P658"/>
       <c r="Q658"/>
       <c r="R658">
@@ -42150,8 +42432,14 @@
       </c>
       <c r="L660"/>
       <c r="M660"/>
-      <c r="N660"/>
-      <c r="O660"/>
+      <c r="N660">
+        <v>91.3</v>
+      </c>
+      <c r="O660" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
       <c r="P660"/>
       <c r="Q660"/>
       <c r="R660">
@@ -44092,8 +44380,14 @@
       </c>
       <c r="L691"/>
       <c r="M691"/>
-      <c r="N691"/>
-      <c r="O691"/>
+      <c r="N691">
+        <v>81.5</v>
+      </c>
+      <c r="O691" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
       <c r="P691"/>
       <c r="Q691"/>
       <c r="R691">
@@ -44224,8 +44518,14 @@
       </c>
       <c r="L693"/>
       <c r="M693"/>
-      <c r="N693"/>
-      <c r="O693"/>
+      <c r="N693">
+        <v>85.8</v>
+      </c>
+      <c r="O693" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
       <c r="P693"/>
       <c r="Q693"/>
       <c r="R693">
@@ -44414,8 +44714,14 @@
       <c r="K696"/>
       <c r="L696"/>
       <c r="M696"/>
-      <c r="N696"/>
-      <c r="O696"/>
+      <c r="N696">
+        <v>94.6</v>
+      </c>
+      <c r="O696" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
       <c r="P696"/>
       <c r="Q696"/>
       <c r="R696">
@@ -44472,8 +44778,14 @@
       <c r="K697"/>
       <c r="L697"/>
       <c r="M697"/>
-      <c r="N697"/>
-      <c r="O697"/>
+      <c r="N697">
+        <v>74.4</v>
+      </c>
+      <c r="O697" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
       <c r="P697"/>
       <c r="Q697"/>
       <c r="R697">
@@ -45364,8 +45676,14 @@
       <c r="K711"/>
       <c r="L711"/>
       <c r="M711"/>
-      <c r="N711"/>
-      <c r="O711"/>
+      <c r="N711">
+        <v>94.1</v>
+      </c>
+      <c r="O711" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
       <c r="P711"/>
       <c r="Q711"/>
       <c r="R711">
@@ -47196,8 +47514,14 @@
       <c r="K739"/>
       <c r="L739"/>
       <c r="M739"/>
-      <c r="N739"/>
-      <c r="O739"/>
+      <c r="N739">
+        <v>80.5</v>
+      </c>
+      <c r="O739" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
       <c r="P739"/>
       <c r="Q739"/>
       <c r="R739">
@@ -48558,8 +48882,14 @@
       </c>
       <c r="L760"/>
       <c r="M760"/>
-      <c r="N760"/>
-      <c r="O760"/>
+      <c r="N760">
+        <v>94.5</v>
+      </c>
+      <c r="O760" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
       <c r="P760"/>
       <c r="Q760"/>
       <c r="R760">
@@ -51266,8 +51596,14 @@
       </c>
       <c r="L802"/>
       <c r="M802"/>
-      <c r="N802"/>
-      <c r="O802"/>
+      <c r="N802">
+        <v>94.3</v>
+      </c>
+      <c r="O802" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
       <c r="P802"/>
       <c r="Q802"/>
       <c r="R802">
@@ -51794,8 +52130,14 @@
       </c>
       <c r="L810"/>
       <c r="M810"/>
-      <c r="N810"/>
-      <c r="O810"/>
+      <c r="N810">
+        <v>87.9</v>
+      </c>
+      <c r="O810" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
       <c r="P810"/>
       <c r="Q810"/>
       <c r="R810">
@@ -55054,8 +55396,14 @@
       <c r="K860"/>
       <c r="L860"/>
       <c r="M860"/>
-      <c r="N860"/>
-      <c r="O860"/>
+      <c r="N860">
+        <v>80.2</v>
+      </c>
+      <c r="O860" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
       <c r="P860"/>
       <c r="Q860"/>
       <c r="R860">
@@ -55302,8 +55650,14 @@
       <c r="K864"/>
       <c r="L864"/>
       <c r="M864"/>
-      <c r="N864"/>
-      <c r="O864"/>
+      <c r="N864">
+        <v>83.5</v>
+      </c>
+      <c r="O864" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
       <c r="P864"/>
       <c r="Q864"/>
       <c r="R864">
@@ -57004,8 +57358,14 @@
       <c r="K891"/>
       <c r="L891"/>
       <c r="M891"/>
-      <c r="N891"/>
-      <c r="O891"/>
+      <c r="N891">
+        <v>87.7</v>
+      </c>
+      <c r="O891" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
       <c r="P891"/>
       <c r="Q891"/>
       <c r="R891">
@@ -58342,8 +58702,14 @@
       </c>
       <c r="L912"/>
       <c r="M912"/>
-      <c r="N912"/>
-      <c r="O912"/>
+      <c r="N912">
+        <v>78.9</v>
+      </c>
+      <c r="O912" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
       <c r="P912"/>
       <c r="Q912"/>
       <c r="R912">
@@ -60432,8 +60798,14 @@
       <c r="K945"/>
       <c r="L945"/>
       <c r="M945"/>
-      <c r="N945"/>
-      <c r="O945"/>
+      <c r="N945">
+        <v>80.0</v>
+      </c>
+      <c r="O945" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
       <c r="P945"/>
       <c r="Q945"/>
       <c r="R945">
@@ -63808,8 +64180,14 @@
       <c r="K997"/>
       <c r="L997"/>
       <c r="M997"/>
-      <c r="N997"/>
-      <c r="O997"/>
+      <c r="N997">
+        <v>93.6</v>
+      </c>
+      <c r="O997" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
       <c r="P997"/>
       <c r="Q997"/>
       <c r="R997">
@@ -66962,8 +67340,14 @@
       <c r="K1046"/>
       <c r="L1046"/>
       <c r="M1046"/>
-      <c r="N1046"/>
-      <c r="O1046"/>
+      <c r="N1046">
+        <v>95.2</v>
+      </c>
+      <c r="O1046" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
       <c r="P1046"/>
       <c r="Q1046"/>
       <c r="R1046">

</xml_diff>